<commit_message>
changes to medicare OBBBA
</commit_message>
<xml_diff>
--- a/results/05-2026/beta/inputs-05-2026.xlsx
+++ b/results/05-2026/beta/inputs-05-2026.xlsx
@@ -4494,7 +4494,7 @@
         <v>0.7</v>
       </c>
       <c r="AH25" t="n">
-        <v>1975.026</v>
+        <v>1993.526</v>
       </c>
       <c r="AI25" t="n">
         <v>344.974</v>
@@ -4545,7 +4545,7 @@
         <v>0.315</v>
       </c>
       <c r="AY25" t="n">
-        <v>1710.213975</v>
+        <v>1714.376475</v>
       </c>
       <c r="AZ25" t="n">
         <v>298.541025</v>
@@ -4652,7 +4652,7 @@
         <v>0.7</v>
       </c>
       <c r="AH26" t="n">
-        <v>2012.824</v>
+        <v>2031.324</v>
       </c>
       <c r="AI26" t="n">
         <v>342.676</v>
@@ -4703,7 +4703,7 @@
         <v>0.315</v>
       </c>
       <c r="AY26" t="n">
-        <v>1755.549675</v>
+        <v>1763.874675</v>
       </c>
       <c r="AZ26" t="n">
         <v>304.437825</v>
@@ -4810,10 +4810,10 @@
         <v>0</v>
       </c>
       <c r="AH27" t="n">
-        <v>2042.95805853092</v>
+        <v>2057.24378921733</v>
       </c>
       <c r="AI27" t="n">
-        <v>348.008366328366</v>
+        <v>352.182603865589</v>
       </c>
       <c r="AJ27" t="n">
         <v>-2956.97812484218</v>
@@ -4861,10 +4861,10 @@
         <v>0.28035</v>
       </c>
       <c r="AY27" t="n">
-        <v>1792.74173816946</v>
+        <v>1804.2810275739</v>
       </c>
       <c r="AZ27" t="n">
-        <v>310.933207423882</v>
+        <v>311.872410869757</v>
       </c>
     </row>
     <row r="28">
@@ -4968,10 +4968,10 @@
         <v>0</v>
       </c>
       <c r="AH28" t="n">
-        <v>2088.12338505647</v>
+        <v>2101.91293984899</v>
       </c>
       <c r="AI28" t="n">
-        <v>353.222696367226</v>
+        <v>357.850955326441</v>
       </c>
       <c r="AJ28" t="n">
         <v>-2989.65648754629</v>
@@ -5019,10 +5019,10 @@
         <v>0.250425</v>
       </c>
       <c r="AY28" t="n">
-        <v>1826.75957480716</v>
+        <v>1841.40151403992</v>
       </c>
       <c r="AZ28" t="n">
-        <v>312.498239106508</v>
+        <v>314.478800818207</v>
       </c>
     </row>
     <row r="29">
@@ -5126,10 +5126,10 @@
         <v>0</v>
       </c>
       <c r="AH29" t="n">
-        <v>2106.59987078557</v>
+        <v>2144.81274540319</v>
       </c>
       <c r="AI29" t="n">
-        <v>355.865936362206</v>
+        <v>366.360153244244</v>
       </c>
       <c r="AJ29" t="n">
         <v>-3025.66274002043</v>
@@ -5177,10 +5177,10 @@
         <v>0.222075</v>
       </c>
       <c r="AY29" t="n">
-        <v>1856.36369573392</v>
+        <v>1875.44103175564</v>
       </c>
       <c r="AZ29" t="n">
-        <v>314.948924788005</v>
+        <v>319.290685298162</v>
       </c>
     </row>
     <row r="30">
@@ -5284,10 +5284,10 @@
         <v>0</v>
       </c>
       <c r="AH30" t="n">
-        <v>2132.08617923157</v>
+        <v>2169.51827816884</v>
       </c>
       <c r="AI30" t="n">
-        <v>356.859779384814</v>
+        <v>366.616641816616</v>
       </c>
       <c r="AJ30" t="n">
         <v>-3082.9686263826</v>
@@ -5335,10 +5335,10 @@
         <v>0.1953</v>
       </c>
       <c r="AY30" t="n">
-        <v>1883.19768606102</v>
+        <v>1906.53474434363</v>
       </c>
       <c r="AZ30" t="n">
-        <v>318.140275149588</v>
+        <v>324.6773297069</v>
       </c>
     </row>
     <row r="31">
@@ -5442,10 +5442,10 @@
         <v>0</v>
       </c>
       <c r="AH31" t="n">
-        <v>2157.0933788699</v>
+        <v>2193.75131366013</v>
       </c>
       <c r="AI31" t="n">
-        <v>358.739093739241</v>
+        <v>367.736414032984</v>
       </c>
       <c r="AJ31" t="n">
         <v>-3129.59282499899</v>
@@ -5493,10 +5493,10 @@
         <v>0.171675</v>
       </c>
       <c r="AY31" t="n">
-        <v>1908.87813313729</v>
+        <v>1937.24893734326</v>
       </c>
       <c r="AZ31" t="n">
-        <v>320.554688817035</v>
+        <v>328.176936994564</v>
       </c>
     </row>
     <row r="32">
@@ -5600,10 +5600,10 @@
         <v>0</v>
       </c>
       <c r="AH32" t="n">
-        <v>2183.90946118689</v>
+        <v>2219.39582271884</v>
       </c>
       <c r="AI32" t="n">
-        <v>360.222346635286</v>
+        <v>368.841811723475</v>
       </c>
       <c r="AJ32" t="n">
         <v>-3156.2442983479</v>
@@ -5651,10 +5651,10 @@
         <v>0.14805</v>
       </c>
       <c r="AY32" t="n">
-        <v>1930.43000026663</v>
+        <v>1963.68258598897</v>
       </c>
       <c r="AZ32" t="n">
-        <v>322.129610127348</v>
+        <v>330.649879683897</v>
       </c>
     </row>
     <row r="33">
@@ -5758,10 +5758,10 @@
         <v>0</v>
       </c>
       <c r="AH33" t="n">
-        <v>2198.34357500005</v>
+        <v>2247.43488963184</v>
       </c>
       <c r="AI33" t="n">
-        <v>367.007979818939</v>
+        <v>382.158253305508</v>
       </c>
       <c r="AJ33" t="n">
         <v>-3179.53643376702</v>
@@ -5809,10 +5809,10 @@
         <v>0.124425</v>
       </c>
       <c r="AY33" t="n">
-        <v>1951.07233371489</v>
+        <v>1986.77256844042</v>
       </c>
       <c r="AZ33" t="n">
-        <v>324.636569905113</v>
+        <v>334.204452197681</v>
       </c>
     </row>
     <row r="34">
@@ -5916,10 +5916,10 @@
         <v>0</v>
       </c>
       <c r="AH34" t="n">
-        <v>2211.92489165399</v>
+        <v>2264.44488252739</v>
       </c>
       <c r="AI34" t="n">
-        <v>375.061936771887</v>
+        <v>390.396915337375</v>
       </c>
       <c r="AJ34" t="n">
         <v>-3214.47999861784</v>
@@ -5967,10 +5967,10 @@
         <v>0.1008</v>
       </c>
       <c r="AY34" t="n">
-        <v>1969.03604400994</v>
+        <v>2008.1310544211</v>
       </c>
       <c r="AZ34" t="n">
-        <v>328.732055317204</v>
+        <v>339.555013739852</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
putting student loans back in (and recovered files)
</commit_message>
<xml_diff>
--- a/results/05-2026/beta/inputs-05-2026.xlsx
+++ b/results/05-2026/beta/inputs-05-2026.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -107,6 +107,9 @@
     <t xml:space="preserve">federal_other_vulnerable_arp</t>
   </si>
   <si>
+    <t xml:space="preserve">federal_student_loans</t>
+  </si>
+  <si>
     <t xml:space="preserve">state_subsidies</t>
   </si>
   <si>
@@ -153,6 +156,9 @@
   </si>
   <si>
     <t xml:space="preserve">post_mpc_federal_other_vulnerable_arp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">post_mpc_federal_student_loans</t>
   </si>
   <si>
     <t xml:space="preserve">post_mpc_state_subsidies</t>
@@ -746,13 +752,19 @@
       <c r="AX1" t="s">
         <v>49</v>
       </c>
+      <c r="AY1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -842,35 +854,35 @@
         <v>0</v>
       </c>
       <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
         <v>0.6</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="AH2" t="n">
         <v>1228.089</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="AI2" t="n">
         <v>183.511</v>
       </c>
-      <c r="AI2" t="n">
+      <c r="AJ2" t="n">
         <v>-1961.394</v>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AK2" t="n">
         <v>-1109.886</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="AL2" t="n">
         <v>-88.1233333333332</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="AM2" t="n">
         <v>-25.3166666666666</v>
       </c>
-      <c r="AM2" t="n">
+      <c r="AN2" t="n">
         <v>1374.885</v>
       </c>
-      <c r="AN2" t="n">
+      <c r="AO2" t="n">
         <v>135.765</v>
       </c>
-      <c r="AO2" t="n">
-        <v>0</v>
-      </c>
       <c r="AP2" t="n">
         <v>0</v>
       </c>
@@ -878,33 +890,39 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
         <v>28.143</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="AT2" t="n">
         <v>30.366</v>
       </c>
-      <c r="AT2" t="n">
-        <v>0</v>
-      </c>
       <c r="AU2" t="n">
         <v>0</v>
       </c>
       <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX2" t="n">
         <v>0.2664</v>
       </c>
-      <c r="AW2" t="n">
+      <c r="AY2" t="n">
         <v>1094.7726</v>
       </c>
-      <c r="AX2" t="n">
+      <c r="AZ2" t="n">
         <v>178.1649</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
@@ -955,7 +973,7 @@
         <v>1797.5</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>199.7</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
@@ -994,69 +1012,75 @@
         <v>0</v>
       </c>
       <c r="AF3" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG3" t="n">
         <v>0.6</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AH3" t="n">
         <v>1326.164</v>
       </c>
-      <c r="AH3" t="n">
+      <c r="AI3" t="n">
         <v>149.436</v>
       </c>
-      <c r="AI3" t="n">
+      <c r="AJ3" t="n">
         <v>-1950.966</v>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AK3" t="n">
         <v>-1107.138</v>
       </c>
-      <c r="AK3" t="n">
-        <v>-80.5999999999999</v>
-      </c>
       <c r="AL3" t="n">
+        <v>-87.2566666666666</v>
+      </c>
+      <c r="AM3" t="n">
         <v>-25.8066666666666</v>
       </c>
-      <c r="AM3" t="n">
+      <c r="AN3" t="n">
         <v>1407.15</v>
       </c>
-      <c r="AN3" t="n">
+      <c r="AO3" t="n">
         <v>137.7225</v>
       </c>
-      <c r="AO3" t="n">
+      <c r="AP3" t="n">
         <v>264.1345</v>
       </c>
-      <c r="AP3" t="n">
-        <v>0</v>
-      </c>
       <c r="AQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="n">
         <v>245.574</v>
       </c>
-      <c r="AR3" t="n">
+      <c r="AS3" t="n">
         <v>73.3005</v>
       </c>
-      <c r="AS3" t="n">
+      <c r="AT3" t="n">
         <v>78.291</v>
       </c>
-      <c r="AT3" t="n">
-        <v>0</v>
-      </c>
       <c r="AU3" t="n">
         <v>0</v>
       </c>
       <c r="AV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>9</v>
+      </c>
+      <c r="AX3" t="n">
         <v>0.2673</v>
       </c>
-      <c r="AW3" t="n">
+      <c r="AY3" t="n">
         <v>1122.5529</v>
       </c>
-      <c r="AX3" t="n">
+      <c r="AZ3" t="n">
         <v>166.7421</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" t="s">
         <v>53</v>
-      </c>
-      <c r="B4" t="s">
-        <v>51</v>
       </c>
       <c r="C4" t="n">
         <v>-1</v>
@@ -1107,7 +1131,7 @@
         <v>1924.5</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>257.7</v>
       </c>
       <c r="T4" t="n">
         <v>0</v>
@@ -1146,69 +1170,75 @@
         <v>0</v>
       </c>
       <c r="AF4" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG4" t="n">
         <v>0.6</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="AH4" t="n">
         <v>1320.282</v>
       </c>
-      <c r="AH4" t="n">
+      <c r="AI4" t="n">
         <v>205.818</v>
       </c>
-      <c r="AI4" t="n">
+      <c r="AJ4" t="n">
         <v>-1957.164</v>
       </c>
-      <c r="AJ4" t="n">
+      <c r="AK4" t="n">
         <v>-1117.866</v>
       </c>
-      <c r="AK4" t="n">
-        <v>-72.5499999999999</v>
-      </c>
       <c r="AL4" t="n">
+        <v>-87.7966666666666</v>
+      </c>
+      <c r="AM4" t="n">
         <v>-26.72</v>
       </c>
-      <c r="AM4" t="n">
+      <c r="AN4" t="n">
         <v>1472.6475</v>
       </c>
-      <c r="AN4" t="n">
+      <c r="AO4" t="n">
         <v>139.9275</v>
       </c>
-      <c r="AO4" t="n">
+      <c r="AP4" t="n">
         <v>117.0225</v>
       </c>
-      <c r="AP4" t="n">
-        <v>0</v>
-      </c>
       <c r="AQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="n">
         <v>462.483</v>
       </c>
-      <c r="AR4" t="n">
+      <c r="AS4" t="n">
         <v>97.3665</v>
       </c>
-      <c r="AS4" t="n">
+      <c r="AT4" t="n">
         <v>126.1278</v>
       </c>
-      <c r="AT4" t="n">
-        <v>0</v>
-      </c>
       <c r="AU4" t="n">
         <v>0</v>
       </c>
       <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>16.65</v>
+      </c>
+      <c r="AX4" t="n">
         <v>0.2682</v>
       </c>
-      <c r="AW4" t="n">
+      <c r="AY4" t="n">
         <v>1145.862</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="AZ4" t="n">
         <v>167.2155</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C5" t="n">
         <v>-1</v>
@@ -1259,7 +1289,7 @@
         <v>1961.9</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>251</v>
       </c>
       <c r="T5" t="n">
         <v>0</v>
@@ -1298,69 +1328,75 @@
         <v>0</v>
       </c>
       <c r="AF5" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG5" t="n">
         <v>0.6</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="AH5" t="n">
         <v>1355.226</v>
       </c>
-      <c r="AH5" t="n">
+      <c r="AI5" t="n">
         <v>171.374</v>
       </c>
-      <c r="AI5" t="n">
+      <c r="AJ5" t="n">
         <v>-1995.864</v>
       </c>
-      <c r="AJ5" t="n">
+      <c r="AK5" t="n">
         <v>-1138.026</v>
       </c>
-      <c r="AK5" t="n">
-        <v>-64.4699999999999</v>
-      </c>
       <c r="AL5" t="n">
+        <v>-88.0833333333332</v>
+      </c>
+      <c r="AM5" t="n">
         <v>-27.51</v>
       </c>
-      <c r="AM5" t="n">
+      <c r="AN5" t="n">
         <v>1510.065</v>
       </c>
-      <c r="AN5" t="n">
+      <c r="AO5" t="n">
         <v>142.3575</v>
       </c>
-      <c r="AO5" t="n">
+      <c r="AP5" t="n">
         <v>63.2366</v>
       </c>
-      <c r="AP5" t="n">
-        <v>0</v>
-      </c>
       <c r="AQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="n">
         <v>366.6105</v>
       </c>
-      <c r="AR5" t="n">
+      <c r="AS5" t="n">
         <v>78.534</v>
       </c>
-      <c r="AS5" t="n">
+      <c r="AT5" t="n">
         <v>138.8241</v>
       </c>
-      <c r="AT5" t="n">
-        <v>0</v>
-      </c>
       <c r="AU5" t="n">
         <v>0</v>
       </c>
       <c r="AV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>23.85</v>
+      </c>
+      <c r="AX5" t="n">
         <v>0.2691</v>
       </c>
-      <c r="AW5" t="n">
+      <c r="AY5" t="n">
         <v>1176.696225</v>
       </c>
-      <c r="AX5" t="n">
+      <c r="AZ5" t="n">
         <v>159.781275</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C6" t="n">
         <v>-1</v>
@@ -1411,7 +1447,7 @@
         <v>2012.3</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>280</v>
       </c>
       <c r="T6" t="n">
         <v>0</v>
@@ -1450,69 +1486,75 @@
         <v>0</v>
       </c>
       <c r="AF6" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG6" t="n">
         <v>2.5</v>
       </c>
-      <c r="AG6" t="n">
+      <c r="AH6" t="n">
         <v>1363.119</v>
       </c>
-      <c r="AH6" t="n">
+      <c r="AI6" t="n">
         <v>205.081</v>
       </c>
-      <c r="AI6" t="n">
+      <c r="AJ6" t="n">
         <v>-2038.506</v>
       </c>
-      <c r="AJ6" t="n">
+      <c r="AK6" t="n">
         <v>-1154.364</v>
       </c>
-      <c r="AK6" t="n">
-        <v>-57.2866666666666</v>
-      </c>
       <c r="AL6" t="n">
+        <v>-90.2333333333332</v>
+      </c>
+      <c r="AM6" t="n">
         <v>-28.4</v>
       </c>
-      <c r="AM6" t="n">
+      <c r="AN6" t="n">
         <v>1595.025</v>
       </c>
-      <c r="AN6" t="n">
+      <c r="AO6" t="n">
         <v>144.99</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="AP6" t="n">
         <v>205.2442</v>
       </c>
-      <c r="AP6" t="n">
+      <c r="AQ6" t="n">
         <v>188.734</v>
       </c>
-      <c r="AQ6" t="n">
+      <c r="AR6" t="n">
         <v>368.9235</v>
       </c>
-      <c r="AR6" t="n">
+      <c r="AS6" t="n">
         <v>78.4215</v>
       </c>
-      <c r="AS6" t="n">
+      <c r="AT6" t="n">
         <v>154.4499</v>
       </c>
-      <c r="AT6" t="n">
-        <v>0</v>
-      </c>
       <c r="AU6" t="n">
         <v>0</v>
       </c>
       <c r="AV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="AX6" t="n">
         <v>0.36405</v>
       </c>
-      <c r="AW6" t="n">
+      <c r="AY6" t="n">
         <v>1207.077975</v>
       </c>
-      <c r="AX6" t="n">
+      <c r="AZ6" t="n">
         <v>164.634525</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C7" t="n">
         <v>-1</v>
@@ -1563,7 +1605,7 @@
         <v>2119.2</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>339.3</v>
       </c>
       <c r="T7" t="n">
         <v>0</v>
@@ -1602,69 +1644,75 @@
         <v>33.92184</v>
       </c>
       <c r="AF7" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG7" t="n">
         <v>8.6</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="AH7" t="n">
         <v>1404.179</v>
       </c>
-      <c r="AH7" t="n">
+      <c r="AI7" t="n">
         <v>220.221</v>
       </c>
-      <c r="AI7" t="n">
+      <c r="AJ7" t="n">
         <v>-2089.86</v>
       </c>
-      <c r="AJ7" t="n">
+      <c r="AK7" t="n">
         <v>-1176.786</v>
       </c>
-      <c r="AK7" t="n">
-        <v>-49.6499999999999</v>
-      </c>
       <c r="AL7" t="n">
+        <v>-93.9066666666666</v>
+      </c>
+      <c r="AM7" t="n">
         <v>-29.7066666666666</v>
       </c>
-      <c r="AM7" t="n">
+      <c r="AN7" t="n">
         <v>1617.542586</v>
       </c>
-      <c r="AN7" t="n">
+      <c r="AO7" t="n">
         <v>147.825</v>
       </c>
-      <c r="AO7" t="n">
+      <c r="AP7" t="n">
         <v>194.0897</v>
       </c>
-      <c r="AP7" t="n">
+      <c r="AQ7" t="n">
         <v>134.81</v>
       </c>
-      <c r="AQ7" t="n">
+      <c r="AR7" t="n">
         <v>379.138</v>
       </c>
-      <c r="AR7" t="n">
+      <c r="AS7" t="n">
         <v>69.91</v>
       </c>
-      <c r="AS7" t="n">
+      <c r="AT7" t="n">
         <v>181.962225</v>
       </c>
-      <c r="AT7" t="n">
+      <c r="AU7" t="n">
         <v>2.3513184</v>
       </c>
-      <c r="AU7" t="n">
+      <c r="AV7" t="n">
         <v>6.78436800000001</v>
       </c>
-      <c r="AV7" t="n">
+      <c r="AW7" t="n">
+        <v>34.65</v>
+      </c>
+      <c r="AX7" t="n">
         <v>0.747225</v>
       </c>
-      <c r="AW7" t="n">
+      <c r="AY7" t="n">
         <v>1224.63135</v>
       </c>
-      <c r="AX7" t="n">
+      <c r="AZ7" t="n">
         <v>180.56115</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C8" t="n">
         <v>-1</v>
@@ -1715,7 +1763,7 @@
         <v>2124.1</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
+        <v>348.7</v>
       </c>
       <c r="T8" t="n">
         <v>0</v>
@@ -1754,69 +1802,75 @@
         <v>44.96616</v>
       </c>
       <c r="AF8" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG8" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG8" t="n">
+      <c r="AH8" t="n">
         <v>1437.905</v>
       </c>
-      <c r="AH8" t="n">
+      <c r="AI8" t="n">
         <v>205.295</v>
       </c>
-      <c r="AI8" t="n">
+      <c r="AJ8" t="n">
         <v>-2144.436</v>
       </c>
-      <c r="AJ8" t="n">
+      <c r="AK8" t="n">
         <v>-1197.36</v>
       </c>
-      <c r="AK8" t="n">
-        <v>-42.1333333333333</v>
-      </c>
       <c r="AL8" t="n">
+        <v>-98.0133333333332</v>
+      </c>
+      <c r="AM8" t="n">
         <v>-31.7766666666666</v>
       </c>
-      <c r="AM8" t="n">
+      <c r="AN8" t="n">
         <v>1643.5143</v>
       </c>
-      <c r="AN8" t="n">
+      <c r="AO8" t="n">
         <v>151.1775</v>
       </c>
-      <c r="AO8" t="n">
+      <c r="AP8" t="n">
         <v>134.3118</v>
       </c>
-      <c r="AP8" t="n">
+      <c r="AQ8" t="n">
         <v>134.81</v>
       </c>
-      <c r="AQ8" t="n">
+      <c r="AR8" t="n">
         <v>328.578</v>
       </c>
-      <c r="AR8" t="n">
+      <c r="AS8" t="n">
         <v>51.465</v>
       </c>
-      <c r="AS8" t="n">
+      <c r="AT8" t="n">
         <v>200.71755</v>
       </c>
-      <c r="AT8" t="n">
+      <c r="AU8" t="n">
         <v>13.06288</v>
       </c>
-      <c r="AU8" t="n">
+      <c r="AV8" t="n">
         <v>14.7599448</v>
       </c>
-      <c r="AV8" t="n">
+      <c r="AW8" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="AX8" t="n">
         <v>0.6939</v>
       </c>
-      <c r="AW8" t="n">
+      <c r="AY8" t="n">
         <v>1251.096525</v>
       </c>
-      <c r="AX8" t="n">
+      <c r="AZ8" t="n">
         <v>180.443475</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C9" t="n">
         <v>-1</v>
@@ -1867,7 +1921,7 @@
         <v>2193.1</v>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
+        <v>374</v>
       </c>
       <c r="T9" t="n">
         <v>0</v>
@@ -1906,69 +1960,75 @@
         <v>52.757</v>
       </c>
       <c r="AF9" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG9" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="AH9" t="n">
         <v>1473.053</v>
       </c>
-      <c r="AH9" t="n">
+      <c r="AI9" t="n">
         <v>182.147</v>
       </c>
-      <c r="AI9" t="n">
+      <c r="AJ9" t="n">
         <v>-2201.688</v>
       </c>
-      <c r="AJ9" t="n">
+      <c r="AK9" t="n">
         <v>-1220.328</v>
       </c>
-      <c r="AK9" t="n">
-        <v>-34.4766666666666</v>
-      </c>
       <c r="AL9" t="n">
+        <v>-102.823333333333</v>
+      </c>
+      <c r="AM9" t="n">
         <v>-35.4366666666666</v>
       </c>
-      <c r="AM9" t="n">
+      <c r="AN9" t="n">
         <v>1691.3997</v>
       </c>
-      <c r="AN9" t="n">
+      <c r="AO9" t="n">
         <v>154.1025</v>
       </c>
-      <c r="AO9" t="n">
+      <c r="AP9" t="n">
         <v>114.6509</v>
       </c>
-      <c r="AP9" t="n">
+      <c r="AQ9" t="n">
         <v>69.393</v>
       </c>
-      <c r="AQ9" t="n">
+      <c r="AR9" t="n">
         <v>272.843</v>
       </c>
-      <c r="AR9" t="n">
+      <c r="AS9" t="n">
         <v>44.17</v>
       </c>
-      <c r="AS9" t="n">
+      <c r="AT9" t="n">
         <v>209.427525</v>
       </c>
-      <c r="AT9" t="n">
+      <c r="AU9" t="n">
         <v>16.12079192</v>
       </c>
-      <c r="AU9" t="n">
+      <c r="AV9" t="n">
         <v>23.6231416</v>
       </c>
-      <c r="AV9" t="n">
+      <c r="AW9" t="n">
+        <v>39.15</v>
+      </c>
+      <c r="AX9" t="n">
         <v>0.6759</v>
       </c>
-      <c r="AW9" t="n">
+      <c r="AY9" t="n">
         <v>1277.6076</v>
       </c>
-      <c r="AX9" t="n">
+      <c r="AZ9" t="n">
         <v>182.8674</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C10" t="n">
         <v>-1</v>
@@ -2019,7 +2079,7 @@
         <v>2285.3</v>
       </c>
       <c r="S10" t="n">
-        <v>0</v>
+        <v>385</v>
       </c>
       <c r="T10" t="n">
         <v>0</v>
@@ -2058,69 +2118,75 @@
         <v>52.757</v>
       </c>
       <c r="AF10" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG10" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG10" t="n">
+      <c r="AH10" t="n">
         <v>1514.338</v>
       </c>
-      <c r="AH10" t="n">
+      <c r="AI10" t="n">
         <v>201.462</v>
       </c>
-      <c r="AI10" t="n">
+      <c r="AJ10" t="n">
         <v>-2296.824</v>
       </c>
-      <c r="AJ10" t="n">
+      <c r="AK10" t="n">
         <v>-1253.778</v>
       </c>
-      <c r="AK10" t="n">
-        <v>-27.8966666666666</v>
-      </c>
       <c r="AL10" t="n">
+        <v>-109.076666666667</v>
+      </c>
+      <c r="AM10" t="n">
         <v>-39.2</v>
       </c>
-      <c r="AM10" t="n">
+      <c r="AN10" t="n">
         <v>1687.3776</v>
       </c>
-      <c r="AN10" t="n">
+      <c r="AO10" t="n">
         <v>156.645</v>
       </c>
-      <c r="AO10" t="n">
+      <c r="AP10" t="n">
         <v>112.7448</v>
       </c>
-      <c r="AP10" t="n">
+      <c r="AQ10" t="n">
         <v>68.825</v>
       </c>
-      <c r="AQ10" t="n">
+      <c r="AR10" t="n">
         <v>218.928</v>
       </c>
-      <c r="AR10" t="n">
+      <c r="AS10" t="n">
         <v>36.383</v>
       </c>
-      <c r="AS10" t="n">
+      <c r="AT10" t="n">
         <v>205.863525</v>
       </c>
-      <c r="AT10" t="n">
+      <c r="AU10" t="n">
         <v>14.371564</v>
       </c>
-      <c r="AU10" t="n">
+      <c r="AV10" t="n">
         <v>31.8029516</v>
       </c>
-      <c r="AV10" t="n">
+      <c r="AW10" t="n">
+        <v>40.95</v>
+      </c>
+      <c r="AX10" t="n">
         <v>0.6534</v>
       </c>
-      <c r="AW10" t="n">
+      <c r="AY10" t="n">
         <v>1311.631875</v>
       </c>
-      <c r="AX10" t="n">
+      <c r="AZ10" t="n">
         <v>182.053125</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C11" t="n">
         <v>-1</v>
@@ -2171,7 +2237,7 @@
         <v>2353.3</v>
       </c>
       <c r="S11" t="n">
-        <v>0</v>
+        <v>425.6</v>
       </c>
       <c r="T11" t="n">
         <v>0</v>
@@ -2210,69 +2276,75 @@
         <v>52.757</v>
       </c>
       <c r="AF11" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG11" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG11" t="n">
+      <c r="AH11" t="n">
         <v>1528.079</v>
       </c>
-      <c r="AH11" t="n">
+      <c r="AI11" t="n">
         <v>224.221</v>
       </c>
-      <c r="AI11" t="n">
+      <c r="AJ11" t="n">
         <v>-2403.36</v>
       </c>
-      <c r="AJ11" t="n">
+      <c r="AK11" t="n">
         <v>-1296.738</v>
       </c>
-      <c r="AK11" t="n">
-        <v>-21.0433333333333</v>
-      </c>
       <c r="AL11" t="n">
+        <v>-116.41</v>
+      </c>
+      <c r="AM11" t="n">
         <v>-42.12</v>
       </c>
-      <c r="AM11" t="n">
+      <c r="AN11" t="n">
         <v>1729.372914</v>
       </c>
-      <c r="AN11" t="n">
+      <c r="AO11" t="n">
         <v>160.065</v>
       </c>
-      <c r="AO11" t="n">
+      <c r="AP11" t="n">
         <v>52.3712</v>
       </c>
-      <c r="AP11" t="n">
+      <c r="AQ11" t="n">
         <v>68.825</v>
       </c>
-      <c r="AQ11" t="n">
+      <c r="AR11" t="n">
         <v>134.724</v>
       </c>
-      <c r="AR11" t="n">
+      <c r="AS11" t="n">
         <v>26.086</v>
       </c>
-      <c r="AS11" t="n">
+      <c r="AT11" t="n">
         <v>196.425675</v>
       </c>
-      <c r="AT11" t="n">
+      <c r="AU11" t="n">
         <v>16.24578</v>
       </c>
-      <c r="AU11" t="n">
+      <c r="AV11" t="n">
         <v>37.7590996</v>
       </c>
-      <c r="AV11" t="n">
+      <c r="AW11" t="n">
+        <v>40.95</v>
+      </c>
+      <c r="AX11" t="n">
         <v>0.621225</v>
       </c>
-      <c r="AW11" t="n">
+      <c r="AY11" t="n">
         <v>1339.509375</v>
       </c>
-      <c r="AX11" t="n">
+      <c r="AZ11" t="n">
         <v>182.953125</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C12" t="n">
         <v>-1</v>
@@ -2323,7 +2395,7 @@
         <v>2270.7</v>
       </c>
       <c r="S12" t="n">
-        <v>0</v>
+        <v>416.9</v>
       </c>
       <c r="T12" t="n">
         <v>4.73961878202226</v>
@@ -2362,69 +2434,75 @@
         <v>52.757</v>
       </c>
       <c r="AF12" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG12" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG12" t="n">
+      <c r="AH12" t="n">
         <v>1557.76</v>
       </c>
-      <c r="AH12" t="n">
+      <c r="AI12" t="n">
         <v>206.14</v>
       </c>
-      <c r="AI12" t="n">
+      <c r="AJ12" t="n">
         <v>-2481.99</v>
       </c>
-      <c r="AJ12" t="n">
+      <c r="AK12" t="n">
         <v>-1316.634</v>
       </c>
-      <c r="AK12" t="n">
-        <v>-14.1466666666667</v>
-      </c>
       <c r="AL12" t="n">
+        <v>-123.41</v>
+      </c>
+      <c r="AM12" t="n">
         <v>-45.3033333333333</v>
       </c>
-      <c r="AM12" t="n">
+      <c r="AN12" t="n">
         <v>1731.3741</v>
       </c>
-      <c r="AN12" t="n">
+      <c r="AO12" t="n">
         <v>166.725</v>
       </c>
-      <c r="AO12" t="n">
+      <c r="AP12" t="n">
         <v>51.4976</v>
       </c>
-      <c r="AP12" t="n">
+      <c r="AQ12" t="n">
         <v>68.115</v>
       </c>
-      <c r="AQ12" t="n">
+      <c r="AR12" t="n">
         <v>76.057</v>
       </c>
-      <c r="AR12" t="n">
+      <c r="AS12" t="n">
         <v>23.248</v>
       </c>
-      <c r="AS12" t="n">
+      <c r="AT12" t="n">
         <v>187.184025</v>
       </c>
-      <c r="AT12" t="n">
+      <c r="AU12" t="n">
         <v>18.119996</v>
       </c>
-      <c r="AU12" t="n">
+      <c r="AV12" t="n">
         <v>41.6178064</v>
       </c>
-      <c r="AV12" t="n">
+      <c r="AW12" t="n">
+        <v>40.95</v>
+      </c>
+      <c r="AX12" t="n">
         <v>0.6246</v>
       </c>
-      <c r="AW12" t="n">
+      <c r="AY12" t="n">
         <v>1366.47675</v>
       </c>
-      <c r="AX12" t="n">
+      <c r="AZ12" t="n">
         <v>183.14325</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C13" t="n">
         <v>-1</v>
@@ -2514,69 +2592,75 @@
         <v>30</v>
       </c>
       <c r="AF13" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG13" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG13" t="n">
+      <c r="AH13" t="n">
         <v>1574.766</v>
       </c>
-      <c r="AH13" t="n">
+      <c r="AI13" t="n">
         <v>220.334</v>
       </c>
-      <c r="AI13" t="n">
+      <c r="AJ13" t="n">
         <v>-2545.866</v>
       </c>
-      <c r="AJ13" t="n">
+      <c r="AK13" t="n">
         <v>-1329.654</v>
       </c>
-      <c r="AK13" t="n">
-        <v>-20.3933333333333</v>
-      </c>
       <c r="AL13" t="n">
+        <v>-129.656666666667</v>
+      </c>
+      <c r="AM13" t="n">
         <v>-48.92</v>
       </c>
-      <c r="AM13" t="n">
+      <c r="AN13" t="n">
         <v>1754.5851</v>
       </c>
-      <c r="AN13" t="n">
+      <c r="AO13" t="n">
         <v>185.1075</v>
       </c>
-      <c r="AO13" t="n">
+      <c r="AP13" t="n">
         <v>51.2176</v>
       </c>
-      <c r="AP13" t="n">
+      <c r="AQ13" t="n">
         <v>68.115</v>
       </c>
-      <c r="AQ13" t="n">
+      <c r="AR13" t="n">
         <v>52.018</v>
       </c>
-      <c r="AR13" t="n">
+      <c r="AS13" t="n">
         <v>22.562</v>
       </c>
-      <c r="AS13" t="n">
+      <c r="AT13" t="n">
         <v>183.625425</v>
       </c>
-      <c r="AT13" t="n">
+      <c r="AU13" t="n">
         <v>16.093332</v>
       </c>
-      <c r="AU13" t="n">
+      <c r="AV13" t="n">
         <v>40.01589</v>
       </c>
-      <c r="AV13" t="n">
+      <c r="AW13" t="n">
+        <v>40.95</v>
+      </c>
+      <c r="AX13" t="n">
         <v>0.627975</v>
       </c>
-      <c r="AW13" t="n">
+      <c r="AY13" t="n">
         <v>1389.362175</v>
       </c>
-      <c r="AX13" t="n">
+      <c r="AZ13" t="n">
         <v>191.735325</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C14" t="n">
         <v>-1</v>
@@ -2666,69 +2750,75 @@
         <v>12</v>
       </c>
       <c r="AF14" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG14" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG14" t="n">
+      <c r="AH14" t="n">
         <v>1626.831</v>
       </c>
-      <c r="AH14" t="n">
+      <c r="AI14" t="n">
         <v>243.069</v>
       </c>
-      <c r="AI14" t="n">
+      <c r="AJ14" t="n">
         <v>-2558.034</v>
       </c>
-      <c r="AJ14" t="n">
+      <c r="AK14" t="n">
         <v>-1342.134</v>
       </c>
-      <c r="AK14" t="n">
-        <v>-27.95</v>
-      </c>
       <c r="AL14" t="n">
+        <v>-137.213333333333</v>
+      </c>
+      <c r="AM14" t="n">
         <v>-52.5999999999999</v>
       </c>
-      <c r="AM14" t="n">
+      <c r="AN14" t="n">
         <v>1774.3536</v>
       </c>
-      <c r="AN14" t="n">
+      <c r="AO14" t="n">
         <v>188.2575</v>
       </c>
-      <c r="AO14" t="n">
+      <c r="AP14" t="n">
         <v>18.424</v>
       </c>
-      <c r="AP14" t="n">
+      <c r="AQ14" t="n">
         <v>68.115</v>
       </c>
-      <c r="AQ14" t="n">
+      <c r="AR14" t="n">
         <v>27.457</v>
       </c>
-      <c r="AR14" t="n">
+      <c r="AS14" t="n">
         <v>21.292</v>
       </c>
-      <c r="AS14" t="n">
+      <c r="AT14" t="n">
         <v>181.097775</v>
       </c>
-      <c r="AT14" t="n">
+      <c r="AU14" t="n">
         <v>14.066668</v>
       </c>
-      <c r="AU14" t="n">
+      <c r="AV14" t="n">
         <v>34.8458316</v>
       </c>
-      <c r="AV14" t="n">
+      <c r="AW14" t="n">
+        <v>40.95</v>
+      </c>
+      <c r="AX14" t="n">
         <v>0.618525</v>
       </c>
-      <c r="AW14" t="n">
+      <c r="AY14" t="n">
         <v>1414.6731</v>
       </c>
-      <c r="AX14" t="n">
+      <c r="AZ14" t="n">
         <v>201.0969</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C15" t="n">
         <v>-1</v>
@@ -2818,69 +2908,75 @@
         <v>12</v>
       </c>
       <c r="AF15" t="n">
+        <v>45</v>
+      </c>
+      <c r="AG15" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG15" t="n">
+      <c r="AH15" t="n">
         <v>1659.996</v>
       </c>
-      <c r="AH15" t="n">
+      <c r="AI15" t="n">
         <v>267.104</v>
       </c>
-      <c r="AI15" t="n">
+      <c r="AJ15" t="n">
         <v>-2564.838</v>
       </c>
-      <c r="AJ15" t="n">
+      <c r="AK15" t="n">
         <v>-1347.348</v>
       </c>
-      <c r="AK15" t="n">
-        <v>-41.8</v>
-      </c>
       <c r="AL15" t="n">
+        <v>-144.406666666667</v>
+      </c>
+      <c r="AM15" t="n">
         <v>-55.9899999999999</v>
       </c>
-      <c r="AM15" t="n">
+      <c r="AN15" t="n">
         <v>1790.19424285714</v>
       </c>
-      <c r="AN15" t="n">
+      <c r="AO15" t="n">
         <v>188.1225</v>
       </c>
-      <c r="AO15" t="n">
+      <c r="AP15" t="n">
         <v>2.1784</v>
       </c>
-      <c r="AP15" t="n">
+      <c r="AQ15" t="n">
         <v>41.153</v>
       </c>
-      <c r="AQ15" t="n">
+      <c r="AR15" t="n">
         <v>9.157</v>
       </c>
-      <c r="AR15" t="n">
+      <c r="AS15" t="n">
         <v>22.948</v>
       </c>
-      <c r="AS15" t="n">
+      <c r="AT15" t="n">
         <v>159.5619</v>
       </c>
-      <c r="AT15" t="n">
+      <c r="AU15" t="n">
         <v>14.28301</v>
       </c>
-      <c r="AU15" t="n">
+      <c r="AV15" t="n">
         <v>28.9760264</v>
       </c>
-      <c r="AV15" t="n">
+      <c r="AW15" t="n">
+        <v>40.95</v>
+      </c>
+      <c r="AX15" t="n">
         <v>0.5679</v>
       </c>
-      <c r="AW15" t="n">
+      <c r="AY15" t="n">
         <v>1444.354425</v>
       </c>
-      <c r="AX15" t="n">
+      <c r="AZ15" t="n">
         <v>210.745575</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C16" t="n">
         <v>-1</v>
@@ -2970,69 +3066,75 @@
         <v>12</v>
       </c>
       <c r="AF16" t="n">
+        <v>2.081508</v>
+      </c>
+      <c r="AG16" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG16" t="n">
+      <c r="AH16" t="n">
         <v>1613.65</v>
       </c>
-      <c r="AH16" t="n">
+      <c r="AI16" t="n">
         <v>290.05</v>
       </c>
-      <c r="AI16" t="n">
+      <c r="AJ16" t="n">
         <v>-2589.162</v>
       </c>
-      <c r="AJ16" t="n">
+      <c r="AK16" t="n">
         <v>-1357.608</v>
       </c>
-      <c r="AK16" t="n">
-        <v>-56.0799999999999</v>
-      </c>
       <c r="AL16" t="n">
+        <v>-150.096666666666</v>
+      </c>
+      <c r="AM16" t="n">
         <v>-58.8866666666666</v>
       </c>
-      <c r="AM16" t="n">
+      <c r="AN16" t="n">
         <v>1810.06238571429</v>
       </c>
-      <c r="AN16" t="n">
+      <c r="AO16" t="n">
         <v>184.0275</v>
       </c>
-      <c r="AO16" t="n">
-        <v>0</v>
-      </c>
       <c r="AP16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ16" t="n">
         <v>41.153</v>
       </c>
-      <c r="AQ16" t="n">
+      <c r="AR16" t="n">
         <v>0.67</v>
       </c>
-      <c r="AR16" t="n">
+      <c r="AS16" t="n">
         <v>26.182</v>
       </c>
-      <c r="AS16" t="n">
+      <c r="AT16" t="n">
         <v>136.667025</v>
       </c>
-      <c r="AT16" t="n">
+      <c r="AU16" t="n">
         <v>14.499352</v>
       </c>
-      <c r="AU16" t="n">
+      <c r="AV16" t="n">
         <v>22.99411</v>
       </c>
-      <c r="AV16" t="n">
+      <c r="AW16" t="n">
+        <v>32.3663016</v>
+      </c>
+      <c r="AX16" t="n">
         <v>0.5706</v>
       </c>
-      <c r="AW16" t="n">
+      <c r="AY16" t="n">
         <v>1456.929675</v>
       </c>
-      <c r="AX16" t="n">
+      <c r="AZ16" t="n">
         <v>229.625325</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C17" t="n">
         <v>-1</v>
@@ -3122,69 +3224,75 @@
         <v>4.222</v>
       </c>
       <c r="AF17" t="n">
+        <v>2.100618</v>
+      </c>
+      <c r="AG17" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG17" t="n">
+      <c r="AH17" t="n">
         <v>1658.388</v>
       </c>
-      <c r="AH17" t="n">
+      <c r="AI17" t="n">
         <v>252.912</v>
       </c>
-      <c r="AI17" t="n">
+      <c r="AJ17" t="n">
         <v>-2609.964</v>
       </c>
-      <c r="AJ17" t="n">
+      <c r="AK17" t="n">
         <v>-1367.988</v>
       </c>
-      <c r="AK17" t="n">
-        <v>-70.8366666666666</v>
-      </c>
       <c r="AL17" t="n">
+        <v>-156.486666666666</v>
+      </c>
+      <c r="AM17" t="n">
         <v>-62.0366666666666</v>
       </c>
-      <c r="AM17" t="n">
+      <c r="AN17" t="n">
         <v>1814.99326071429</v>
       </c>
-      <c r="AN17" t="n">
+      <c r="AO17" t="n">
         <v>168.84</v>
       </c>
-      <c r="AO17" t="n">
-        <v>0</v>
-      </c>
       <c r="AP17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ17" t="n">
         <v>41.153</v>
       </c>
-      <c r="AQ17" t="n">
+      <c r="AR17" t="n">
         <v>0.174</v>
       </c>
-      <c r="AR17" t="n">
+      <c r="AS17" t="n">
         <v>28.155</v>
       </c>
-      <c r="AS17" t="n">
+      <c r="AT17" t="n">
         <v>126.927</v>
       </c>
-      <c r="AT17" t="n">
+      <c r="AU17" t="n">
         <v>14.261254</v>
       </c>
-      <c r="AU17" t="n">
+      <c r="AV17" t="n">
         <v>16.69038</v>
       </c>
-      <c r="AV17" t="n">
+      <c r="AW17" t="n">
+        <v>25.07397996</v>
+      </c>
+      <c r="AX17" t="n">
         <v>0.5733</v>
       </c>
-      <c r="AW17" t="n">
+      <c r="AY17" t="n">
         <v>1475.744625</v>
       </c>
-      <c r="AX17" t="n">
+      <c r="AZ17" t="n">
         <v>236.955375</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C18" t="n">
         <v>-1</v>
@@ -3274,69 +3382,75 @@
         <v>4.222</v>
       </c>
       <c r="AF18" t="n">
+        <v>2.58153</v>
+      </c>
+      <c r="AG18" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG18" t="n">
+      <c r="AH18" t="n">
         <v>1680.381</v>
       </c>
-      <c r="AH18" t="n">
+      <c r="AI18" t="n">
         <v>298.119</v>
       </c>
-      <c r="AI18" t="n">
+      <c r="AJ18" t="n">
         <v>-2614.512</v>
       </c>
-      <c r="AJ18" t="n">
+      <c r="AK18" t="n">
         <v>-1373.712</v>
       </c>
-      <c r="AK18" t="n">
-        <v>-86.5799999999999</v>
-      </c>
       <c r="AL18" t="n">
+        <v>-162.896666666666</v>
+      </c>
+      <c r="AM18" t="n">
         <v>-65.0899999999999</v>
       </c>
-      <c r="AM18" t="n">
+      <c r="AN18" t="n">
         <v>1840.44413571429</v>
       </c>
-      <c r="AN18" t="n">
+      <c r="AO18" t="n">
         <v>169.65</v>
       </c>
-      <c r="AO18" t="n">
-        <v>0</v>
-      </c>
       <c r="AP18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ18" t="n">
         <v>34.1285</v>
       </c>
-      <c r="AQ18" t="n">
+      <c r="AR18" t="n">
         <v>0.08</v>
       </c>
-      <c r="AR18" t="n">
+      <c r="AS18" t="n">
         <v>29.581</v>
       </c>
-      <c r="AS18" t="n">
+      <c r="AT18" t="n">
         <v>118.68525</v>
       </c>
-      <c r="AT18" t="n">
+      <c r="AU18" t="n">
         <v>14.023156</v>
       </c>
-      <c r="AU18" t="n">
+      <c r="AV18" t="n">
         <v>12.61027</v>
       </c>
-      <c r="AV18" t="n">
+      <c r="AW18" t="n">
+        <v>18.30645234</v>
+      </c>
+      <c r="AX18" t="n">
         <v>0.5418</v>
       </c>
-      <c r="AW18" t="n">
+      <c r="AY18" t="n">
         <v>1487.793375</v>
       </c>
-      <c r="AX18" t="n">
+      <c r="AZ18" t="n">
         <v>249.341625</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C19" t="n">
         <v>-1</v>
@@ -3426,69 +3540,75 @@
         <v>4.222</v>
       </c>
       <c r="AF19" t="n">
+        <v>2.604045</v>
+      </c>
+      <c r="AG19" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG19" t="n">
+      <c r="AH19" t="n">
         <v>1707.978</v>
       </c>
-      <c r="AH19" t="n">
+      <c r="AI19" t="n">
         <v>314.922</v>
       </c>
-      <c r="AI19" t="n">
+      <c r="AJ19" t="n">
         <v>-2622.426</v>
       </c>
-      <c r="AJ19" t="n">
+      <c r="AK19" t="n">
         <v>-1378.08</v>
       </c>
-      <c r="AK19" t="n">
-        <v>-103.09</v>
-      </c>
       <c r="AL19" t="n">
+        <v>-168.096666666666</v>
+      </c>
+      <c r="AM19" t="n">
         <v>-67.4566666666666</v>
       </c>
-      <c r="AM19" t="n">
+      <c r="AN19" t="n">
         <v>1875.22286785714</v>
       </c>
-      <c r="AN19" t="n">
+      <c r="AO19" t="n">
         <v>173.115</v>
       </c>
-      <c r="AO19" t="n">
-        <v>0</v>
-      </c>
       <c r="AP19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ19" t="n">
         <v>27.388</v>
       </c>
-      <c r="AQ19" t="n">
+      <c r="AR19" t="n">
         <v>0.035</v>
       </c>
-      <c r="AR19" t="n">
+      <c r="AS19" t="n">
         <v>30.805</v>
       </c>
-      <c r="AS19" t="n">
+      <c r="AT19" t="n">
         <v>96.491025</v>
       </c>
-      <c r="AT19" t="n">
+      <c r="AU19" t="n">
         <v>13.04705068</v>
       </c>
-      <c r="AU19" t="n">
+      <c r="AV19" t="n">
         <v>9.32794</v>
       </c>
-      <c r="AV19" t="n">
+      <c r="AW19" t="n">
+        <v>11.95799418</v>
+      </c>
+      <c r="AX19" t="n">
         <v>0.4005</v>
       </c>
-      <c r="AW19" t="n">
+      <c r="AY19" t="n">
         <v>1498.589325</v>
       </c>
-      <c r="AX19" t="n">
+      <c r="AZ19" t="n">
         <v>260.100675</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C20" t="n">
         <v>-1</v>
@@ -3578,69 +3698,75 @@
         <v>4.222</v>
       </c>
       <c r="AF20" t="n">
+        <v>2.8036115</v>
+      </c>
+      <c r="AG20" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG20" t="n">
+      <c r="AH20" t="n">
         <v>1744.359</v>
       </c>
-      <c r="AH20" t="n">
+      <c r="AI20" t="n">
         <v>315.441</v>
       </c>
-      <c r="AI20" t="n">
+      <c r="AJ20" t="n">
         <v>-2629.842</v>
       </c>
-      <c r="AJ20" t="n">
+      <c r="AK20" t="n">
         <v>-1390.32</v>
       </c>
-      <c r="AK20" t="n">
-        <v>-119.443333333333</v>
-      </c>
       <c r="AL20" t="n">
+        <v>-172.826666666666</v>
+      </c>
+      <c r="AM20" t="n">
         <v>-69.0033333333332</v>
       </c>
-      <c r="AM20" t="n">
+      <c r="AN20" t="n">
         <v>1912.3191</v>
       </c>
-      <c r="AN20" t="n">
+      <c r="AO20" t="n">
         <v>178.3125</v>
       </c>
-      <c r="AO20" t="n">
-        <v>0</v>
-      </c>
       <c r="AP20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ20" t="n">
         <v>20.6475</v>
       </c>
-      <c r="AQ20" t="n">
+      <c r="AR20" t="n">
         <v>0.012</v>
       </c>
-      <c r="AR20" t="n">
+      <c r="AS20" t="n">
         <v>31.843</v>
       </c>
-      <c r="AS20" t="n">
+      <c r="AT20" t="n">
         <v>75.838725</v>
       </c>
-      <c r="AT20" t="n">
+      <c r="AU20" t="n">
         <v>8.517842</v>
       </c>
-      <c r="AU20" t="n">
+      <c r="AV20" t="n">
         <v>6.35096</v>
       </c>
-      <c r="AV20" t="n">
+      <c r="AW20" t="n">
+        <v>8.21888317</v>
+      </c>
+      <c r="AX20" t="n">
         <v>0.4014</v>
       </c>
-      <c r="AW20" t="n">
+      <c r="AY20" t="n">
         <v>1527.99885</v>
       </c>
-      <c r="AX20" t="n">
+      <c r="AZ20" t="n">
         <v>265.81365</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C21" t="n">
         <v>-1</v>
@@ -3730,69 +3856,75 @@
         <v>2.372</v>
       </c>
       <c r="AF21" t="n">
+        <v>2.833394</v>
+      </c>
+      <c r="AG21" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG21" t="n">
+      <c r="AH21" t="n">
         <v>1786.697</v>
       </c>
-      <c r="AH21" t="n">
+      <c r="AI21" t="n">
         <v>314.303</v>
       </c>
-      <c r="AI21" t="n">
+      <c r="AJ21" t="n">
         <v>-2642.622</v>
       </c>
-      <c r="AJ21" t="n">
+      <c r="AK21" t="n">
         <v>-1404.93</v>
       </c>
-      <c r="AK21" t="n">
-        <v>-136.396666666667</v>
-      </c>
       <c r="AL21" t="n">
+        <v>-177.313333333333</v>
+      </c>
+      <c r="AM21" t="n">
         <v>-69.0299999999999</v>
       </c>
-      <c r="AM21" t="n">
+      <c r="AN21" t="n">
         <v>1954.416375</v>
       </c>
-      <c r="AN21" t="n">
+      <c r="AO21" t="n">
         <v>181.6425</v>
       </c>
-      <c r="AO21" t="n">
-        <v>0</v>
-      </c>
       <c r="AP21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ21" t="n">
         <v>13.836</v>
       </c>
-      <c r="AQ21" t="n">
-        <v>0</v>
-      </c>
       <c r="AR21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS21" t="n">
         <v>32.631</v>
       </c>
-      <c r="AS21" t="n">
+      <c r="AT21" t="n">
         <v>65.877975</v>
       </c>
-      <c r="AT21" t="n">
+      <c r="AU21" t="n">
         <v>6.576191</v>
       </c>
-      <c r="AU21" t="n">
+      <c r="AV21" t="n">
         <v>4.56094</v>
       </c>
-      <c r="AV21" t="n">
+      <c r="AW21" t="n">
+        <v>6.190300475</v>
+      </c>
+      <c r="AX21" t="n">
         <v>0.4023</v>
       </c>
-      <c r="AW21" t="n">
+      <c r="AY21" t="n">
         <v>1556.868375</v>
       </c>
-      <c r="AX21" t="n">
+      <c r="AZ21" t="n">
         <v>279.626625</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C22" t="n">
         <v>-1</v>
@@ -3882,69 +4014,75 @@
         <v>2.372</v>
       </c>
       <c r="AF22" t="n">
+        <v>2.8239574</v>
+      </c>
+      <c r="AG22" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG22" t="n">
+      <c r="AH22" t="n">
         <v>1811.332</v>
       </c>
-      <c r="AH22" t="n">
+      <c r="AI22" t="n">
         <v>316.468</v>
       </c>
-      <c r="AI22" t="n">
+      <c r="AJ22" t="n">
         <v>-2684.838</v>
       </c>
-      <c r="AJ22" t="n">
+      <c r="AK22" t="n">
         <v>-1421.406</v>
       </c>
-      <c r="AK22" t="n">
-        <v>-152.036666666667</v>
-      </c>
       <c r="AL22" t="n">
+        <v>-180.12</v>
+      </c>
+      <c r="AM22" t="n">
         <v>-69.0199999999999</v>
       </c>
-      <c r="AM22" t="n">
+      <c r="AN22" t="n">
         <v>1995.11865</v>
       </c>
-      <c r="AN22" t="n">
+      <c r="AO22" t="n">
         <v>183.555</v>
       </c>
-      <c r="AO22" t="n">
-        <v>0</v>
-      </c>
       <c r="AP22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ22" t="n">
         <v>7.0245</v>
       </c>
-      <c r="AQ22" t="n">
-        <v>0</v>
-      </c>
       <c r="AR22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS22" t="n">
         <v>33.123</v>
       </c>
-      <c r="AS22" t="n">
+      <c r="AT22" t="n">
         <v>61.47135</v>
       </c>
-      <c r="AT22" t="n">
+      <c r="AU22" t="n">
         <v>4.63454</v>
       </c>
-      <c r="AU22" t="n">
+      <c r="AV22" t="n">
         <v>3.85754</v>
       </c>
-      <c r="AV22" t="n">
+      <c r="AW22" t="n">
+        <v>4.12709705</v>
+      </c>
+      <c r="AX22" t="n">
         <v>0.3861</v>
       </c>
-      <c r="AW22" t="n">
+      <c r="AY22" t="n">
         <v>1586.33235</v>
       </c>
-      <c r="AX22" t="n">
+      <c r="AZ22" t="n">
         <v>283.75515</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C23" t="n">
         <v>-1</v>
@@ -4034,69 +4172,75 @@
         <v>2.372</v>
       </c>
       <c r="AF23" t="n">
+        <v>2.8656558</v>
+      </c>
+      <c r="AG23" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG23" t="n">
+      <c r="AH23" t="n">
         <v>1877.66</v>
       </c>
-      <c r="AH23" t="n">
+      <c r="AI23" t="n">
         <v>319.14</v>
       </c>
-      <c r="AI23" t="n">
+      <c r="AJ23" t="n">
         <v>-2747.832</v>
       </c>
-      <c r="AJ23" t="n">
+      <c r="AK23" t="n">
         <v>-1439.904</v>
       </c>
-      <c r="AK23" t="n">
-        <v>-167.693333333333</v>
-      </c>
       <c r="AL23" t="n">
+        <v>-181.59</v>
+      </c>
+      <c r="AM23" t="n">
         <v>-69.6399999999999</v>
       </c>
-      <c r="AM23" t="n">
+      <c r="AN23" t="n">
         <v>2051.075925</v>
       </c>
-      <c r="AN23" t="n">
+      <c r="AO23" t="n">
         <v>184.5225</v>
       </c>
-      <c r="AO23" t="n">
-        <v>0</v>
-      </c>
       <c r="AP23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ23" t="n">
         <v>0.213</v>
       </c>
-      <c r="AQ23" t="n">
-        <v>0</v>
-      </c>
       <c r="AR23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS23" t="n">
         <v>33.62</v>
       </c>
-      <c r="AS23" t="n">
+      <c r="AT23" t="n">
         <v>55.2555</v>
       </c>
-      <c r="AT23" t="n">
+      <c r="AU23" t="n">
         <v>2.745007</v>
       </c>
-      <c r="AU23" t="n">
+      <c r="AV23" t="n">
         <v>3.17264</v>
       </c>
-      <c r="AV23" t="n">
+      <c r="AW23" t="n">
+        <v>2.478820453</v>
+      </c>
+      <c r="AX23" t="n">
         <v>0.315</v>
       </c>
-      <c r="AW23" t="n">
+      <c r="AY23" t="n">
         <v>1624.5108</v>
       </c>
-      <c r="AX23" t="n">
+      <c r="AZ23" t="n">
         <v>284.7042</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C24" t="n">
         <v>-1</v>
@@ -4186,69 +4330,75 @@
         <v>2.372</v>
       </c>
       <c r="AF24" t="n">
+        <v>-8.076788</v>
+      </c>
+      <c r="AG24" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG24" t="n">
+      <c r="AH24" t="n">
         <v>1936.933</v>
       </c>
-      <c r="AH24" t="n">
+      <c r="AI24" t="n">
         <v>346.267</v>
       </c>
-      <c r="AI24" t="n">
+      <c r="AJ24" t="n">
         <v>-2818.38</v>
       </c>
-      <c r="AJ24" t="n">
+      <c r="AK24" t="n">
         <v>-1458.912</v>
       </c>
-      <c r="AK24" t="n">
+      <c r="AL24" t="n">
         <v>-174.643333333333</v>
       </c>
-      <c r="AL24" t="n">
+      <c r="AM24" t="n">
         <v>-69.5433333333333</v>
       </c>
-      <c r="AM24" t="n">
+      <c r="AN24" t="n">
         <v>2093.9607</v>
       </c>
-      <c r="AN24" t="n">
+      <c r="AO24" t="n">
         <v>183.3975</v>
       </c>
-      <c r="AO24" t="n">
-        <v>0</v>
-      </c>
       <c r="AP24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ24" t="n">
         <v>0.142</v>
       </c>
-      <c r="AQ24" t="n">
-        <v>0</v>
-      </c>
       <c r="AR24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS24" t="n">
         <v>34.021</v>
       </c>
-      <c r="AS24" t="n">
+      <c r="AT24" t="n">
         <v>50.655375</v>
       </c>
-      <c r="AT24" t="n">
+      <c r="AU24" t="n">
         <v>0.855474</v>
       </c>
-      <c r="AU24" t="n">
+      <c r="AV24" t="n">
         <v>2.58402</v>
       </c>
-      <c r="AV24" t="n">
+      <c r="AW24" t="n">
+        <v>0.344274675</v>
+      </c>
+      <c r="AX24" t="n">
         <v>0.315</v>
       </c>
-      <c r="AW24" t="n">
+      <c r="AY24" t="n">
         <v>1667.83995</v>
       </c>
-      <c r="AX24" t="n">
+      <c r="AZ24" t="n">
         <v>291.64005</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C25" t="n">
         <v>-1</v>
@@ -4338,69 +4488,75 @@
         <v>0.49</v>
       </c>
       <c r="AF25" t="n">
+        <v>-8.046285</v>
+      </c>
+      <c r="AG25" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG25" t="n">
+      <c r="AH25" t="n">
         <v>1975.026</v>
       </c>
-      <c r="AH25" t="n">
+      <c r="AI25" t="n">
         <v>344.974</v>
       </c>
-      <c r="AI25" t="n">
+      <c r="AJ25" t="n">
         <v>-2881.752</v>
       </c>
-      <c r="AJ25" t="n">
+      <c r="AK25" t="n">
         <v>-1479.648</v>
       </c>
-      <c r="AK25" t="n">
+      <c r="AL25" t="n">
         <v>-175.923893795779</v>
       </c>
-      <c r="AL25" t="n">
+      <c r="AM25" t="n">
         <v>-69.7933333333333</v>
       </c>
-      <c r="AM25" t="n">
+      <c r="AN25" t="n">
         <v>2130.824925</v>
       </c>
-      <c r="AN25" t="n">
+      <c r="AO25" t="n">
         <v>183.69</v>
       </c>
-      <c r="AO25" t="n">
-        <v>0</v>
-      </c>
       <c r="AP25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ25" t="n">
         <v>0.071</v>
       </c>
-      <c r="AQ25" t="n">
-        <v>0</v>
-      </c>
       <c r="AR25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS25" t="n">
         <v>34.282</v>
       </c>
-      <c r="AS25" t="n">
+      <c r="AT25" t="n">
         <v>47.119725</v>
       </c>
-      <c r="AT25" t="n">
+      <c r="AU25" t="n">
         <v>0.573855</v>
       </c>
-      <c r="AU25" t="n">
+      <c r="AV25" t="n">
         <v>2.04112</v>
       </c>
-      <c r="AV25" t="n">
+      <c r="AW25" t="n">
+        <v>-1.471562937</v>
+      </c>
+      <c r="AX25" t="n">
         <v>0.315</v>
       </c>
-      <c r="AW25" t="n">
+      <c r="AY25" t="n">
         <v>1710.213975</v>
       </c>
-      <c r="AX25" t="n">
+      <c r="AZ25" t="n">
         <v>298.541025</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C26" t="n">
         <v>-1</v>
@@ -4490,35 +4646,35 @@
         <v>0</v>
       </c>
       <c r="AF26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG26" t="n">
         <v>0.7</v>
       </c>
-      <c r="AG26" t="n">
+      <c r="AH26" t="n">
         <v>2012.824</v>
       </c>
-      <c r="AH26" t="n">
+      <c r="AI26" t="n">
         <v>336.776</v>
       </c>
-      <c r="AI26" t="n">
+      <c r="AJ26" t="n">
         <v>-2922.108</v>
       </c>
-      <c r="AJ26" t="n">
+      <c r="AK26" t="n">
         <v>-1500.174</v>
       </c>
-      <c r="AK26" t="n">
+      <c r="AL26" t="n">
         <v>-176.784596300125</v>
       </c>
-      <c r="AL26" t="n">
+      <c r="AM26" t="n">
         <v>-70.4366666666666</v>
       </c>
-      <c r="AM26" t="n">
+      <c r="AN26" t="n">
         <v>2148.757875</v>
       </c>
-      <c r="AN26" t="n">
+      <c r="AO26" t="n">
         <v>183.7575</v>
       </c>
-      <c r="AO26" t="n">
-        <v>0</v>
-      </c>
       <c r="AP26" t="n">
         <v>0</v>
       </c>
@@ -4526,33 +4682,39 @@
         <v>0</v>
       </c>
       <c r="AR26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS26" t="n">
         <v>34.149</v>
       </c>
-      <c r="AS26" t="n">
+      <c r="AT26" t="n">
         <v>48.21165</v>
       </c>
-      <c r="AT26" t="n">
+      <c r="AU26" t="n">
         <v>0.378236</v>
       </c>
-      <c r="AU26" t="n">
+      <c r="AV26" t="n">
         <v>1.53068</v>
       </c>
-      <c r="AV26" t="n">
+      <c r="AW26" t="n">
+        <v>-1.590137919</v>
+      </c>
+      <c r="AX26" t="n">
         <v>0.315</v>
       </c>
-      <c r="AW26" t="n">
+      <c r="AY26" t="n">
         <v>1755.549675</v>
       </c>
-      <c r="AX26" t="n">
+      <c r="AZ26" t="n">
         <v>303.110325</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -4645,32 +4807,32 @@
         <v>0</v>
       </c>
       <c r="AG27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH27" t="n">
         <v>2034.15648172719</v>
       </c>
-      <c r="AH27" t="n">
+      <c r="AI27" t="n">
         <v>342.239043840667</v>
       </c>
-      <c r="AI27" t="n">
+      <c r="AJ27" t="n">
         <v>-2948.09633521465</v>
       </c>
-      <c r="AJ27" t="n">
+      <c r="AK27" t="n">
         <v>-1520.25372972477</v>
       </c>
-      <c r="AK27" t="n">
+      <c r="AL27" t="n">
         <v>-167.357178947116</v>
       </c>
-      <c r="AL27" t="n">
+      <c r="AM27" t="n">
         <v>-71.1356391763352</v>
       </c>
-      <c r="AM27" t="n">
+      <c r="AN27" t="n">
         <v>2148.5514816375</v>
       </c>
-      <c r="AN27" t="n">
+      <c r="AO27" t="n">
         <v>183.84490125</v>
       </c>
-      <c r="AO27" t="n">
-        <v>0</v>
-      </c>
       <c r="AP27" t="n">
         <v>0</v>
       </c>
@@ -4678,33 +4840,39 @@
         <v>0</v>
       </c>
       <c r="AR27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS27" t="n">
         <v>33.851</v>
       </c>
-      <c r="AS27" t="n">
+      <c r="AT27" t="n">
         <v>49.2903</v>
       </c>
-      <c r="AT27" t="n">
+      <c r="AU27" t="n">
         <v>0.211344</v>
       </c>
-      <c r="AU27" t="n">
+      <c r="AV27" t="n">
         <v>1.05376</v>
       </c>
-      <c r="AV27" t="n">
+      <c r="AW27" t="n">
+        <v>-1.846002748</v>
+      </c>
+      <c r="AX27" t="n">
         <v>0.28035</v>
       </c>
-      <c r="AW27" t="n">
+      <c r="AY27" t="n">
         <v>1790.76138338862</v>
       </c>
-      <c r="AX27" t="n">
+      <c r="AZ27" t="n">
         <v>308.30760986415</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -4797,32 +4965,32 @@
         <v>0</v>
       </c>
       <c r="AG28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH28" t="n">
         <v>2079.06393824034</v>
       </c>
-      <c r="AH28" t="n">
+      <c r="AI28" t="n">
         <v>346.915782596978</v>
       </c>
-      <c r="AI28" t="n">
+      <c r="AJ28" t="n">
         <v>-2978.81489909456</v>
       </c>
-      <c r="AJ28" t="n">
+      <c r="AK28" t="n">
         <v>-1540.10527694422</v>
       </c>
-      <c r="AK28" t="n">
+      <c r="AL28" t="n">
         <v>-157.377091960497</v>
       </c>
-      <c r="AL28" t="n">
+      <c r="AM28" t="n">
         <v>-71.9136604996341</v>
       </c>
-      <c r="AM28" t="n">
+      <c r="AN28" t="n">
         <v>2162.28213508865</v>
       </c>
-      <c r="AN28" t="n">
+      <c r="AO28" t="n">
         <v>183.934489753125</v>
       </c>
-      <c r="AO28" t="n">
-        <v>0</v>
-      </c>
       <c r="AP28" t="n">
         <v>0</v>
       </c>
@@ -4830,33 +4998,39 @@
         <v>0</v>
       </c>
       <c r="AR28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS28" t="n">
         <v>33.49</v>
       </c>
-      <c r="AS28" t="n">
+      <c r="AT28" t="n">
         <v>50.3919</v>
       </c>
-      <c r="AT28" t="n">
+      <c r="AU28" t="n">
         <v>-0.00499800000000003</v>
       </c>
-      <c r="AU28" t="n">
+      <c r="AV28" t="n">
         <v>0.61906</v>
       </c>
-      <c r="AV28" t="n">
+      <c r="AW28" t="n">
+        <v>-1.53603725</v>
+      </c>
+      <c r="AX28" t="n">
         <v>0.250425</v>
       </c>
-      <c r="AW28" t="n">
+      <c r="AY28" t="n">
         <v>1822.74084449269</v>
       </c>
-      <c r="AX28" t="n">
+      <c r="AZ28" t="n">
         <v>308.45358594847</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
+        <v>81</v>
+      </c>
+      <c r="B29" t="s">
         <v>79</v>
-      </c>
-      <c r="B29" t="s">
-        <v>77</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
@@ -4949,32 +5123,32 @@
         <v>0</v>
       </c>
       <c r="AG29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH29" t="n">
         <v>2097.81586073649</v>
       </c>
-      <c r="AH29" t="n">
+      <c r="AI29" t="n">
         <v>349.124163683446</v>
       </c>
-      <c r="AI29" t="n">
+      <c r="AJ29" t="n">
         <v>-3012.85618416554</v>
       </c>
-      <c r="AJ29" t="n">
+      <c r="AK29" t="n">
         <v>-1558.86126701323</v>
       </c>
-      <c r="AK29" t="n">
+      <c r="AL29" t="n">
         <v>-157.801071173951</v>
       </c>
-      <c r="AL29" t="n">
+      <c r="AM29" t="n">
         <v>-72.589714644089</v>
       </c>
-      <c r="AM29" t="n">
+      <c r="AN29" t="n">
         <v>2179.42362267636</v>
       </c>
-      <c r="AN29" t="n">
+      <c r="AO29" t="n">
         <v>183.779052227508</v>
       </c>
-      <c r="AO29" t="n">
-        <v>0</v>
-      </c>
       <c r="AP29" t="n">
         <v>0</v>
       </c>
@@ -4982,33 +5156,39 @@
         <v>0</v>
       </c>
       <c r="AR29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS29" t="n">
         <v>33.137</v>
       </c>
-      <c r="AS29" t="n">
+      <c r="AT29" t="n">
         <v>51.689025</v>
       </c>
-      <c r="AT29" t="n">
+      <c r="AU29" t="n">
         <v>-0.028203</v>
       </c>
-      <c r="AU29" t="n">
+      <c r="AV29" t="n">
         <v>0.37618</v>
       </c>
-      <c r="AV29" t="n">
+      <c r="AW29" t="n">
+        <v>-0.871763964</v>
+      </c>
+      <c r="AX29" t="n">
         <v>0.222075</v>
       </c>
-      <c r="AW29" t="n">
+      <c r="AY29" t="n">
         <v>1850.3685631584</v>
       </c>
-      <c r="AX29" t="n">
+      <c r="AZ29" t="n">
         <v>309.387372777245</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
@@ -5101,32 +5281,32 @@
         <v>0</v>
       </c>
       <c r="AG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH30" t="n">
         <v>2123.58948418872</v>
       </c>
-      <c r="AH30" t="n">
+      <c r="AI30" t="n">
         <v>349.670052964896</v>
       </c>
-      <c r="AI30" t="n">
+      <c r="AJ30" t="n">
         <v>-3068.05990223096</v>
       </c>
-      <c r="AJ30" t="n">
+      <c r="AK30" t="n">
         <v>-1577.48682791785</v>
       </c>
-      <c r="AK30" t="n">
+      <c r="AL30" t="n">
         <v>-157.380294989923</v>
       </c>
-      <c r="AL30" t="n">
+      <c r="AM30" t="n">
         <v>-73.2304222849377</v>
       </c>
-      <c r="AM30" t="n">
+      <c r="AN30" t="n">
         <v>2204.78475886786</v>
       </c>
-      <c r="AN30" t="n">
+      <c r="AO30" t="n">
         <v>184.188876108077</v>
       </c>
-      <c r="AO30" t="n">
-        <v>0</v>
-      </c>
       <c r="AP30" t="n">
         <v>0</v>
       </c>
@@ -5134,33 +5314,39 @@
         <v>0</v>
       </c>
       <c r="AR30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS30" t="n">
         <v>33.112</v>
       </c>
-      <c r="AS30" t="n">
+      <c r="AT30" t="n">
         <v>52.8453</v>
       </c>
-      <c r="AT30" t="n">
+      <c r="AU30" t="n">
         <v>-0.051408</v>
       </c>
-      <c r="AU30" t="n">
+      <c r="AV30" t="n">
         <v>0.23798</v>
       </c>
-      <c r="AV30" t="n">
+      <c r="AW30" t="n">
+        <v>-0.691527418</v>
+      </c>
+      <c r="AX30" t="n">
         <v>0.1953</v>
       </c>
-      <c r="AW30" t="n">
+      <c r="AY30" t="n">
         <v>1875.29079710087</v>
       </c>
-      <c r="AX30" t="n">
+      <c r="AZ30" t="n">
         <v>312.288534694347</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
@@ -5253,32 +5439,32 @@
         <v>0</v>
       </c>
       <c r="AG31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH31" t="n">
         <v>2147.9873262361</v>
       </c>
-      <c r="AH31" t="n">
+      <c r="AI31" t="n">
         <v>351.996686355047</v>
       </c>
-      <c r="AI31" t="n">
+      <c r="AJ31" t="n">
         <v>-3112.56903978137</v>
       </c>
-      <c r="AJ31" t="n">
+      <c r="AK31" t="n">
         <v>-1595.68266791584</v>
       </c>
-      <c r="AK31" t="n">
+      <c r="AL31" t="n">
         <v>-156.336090019183</v>
       </c>
-      <c r="AL31" t="n">
+      <c r="AM31" t="n">
         <v>-73.9606574683808</v>
       </c>
-      <c r="AM31" t="n">
+      <c r="AN31" t="n">
         <v>2229.81990911763</v>
       </c>
-      <c r="AN31" t="n">
+      <c r="AO31" t="n">
         <v>184.649348298347</v>
       </c>
-      <c r="AO31" t="n">
-        <v>0</v>
-      </c>
       <c r="AP31" t="n">
         <v>0</v>
       </c>
@@ -5286,33 +5472,39 @@
         <v>0</v>
       </c>
       <c r="AR31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS31" t="n">
         <v>33.334</v>
       </c>
-      <c r="AS31" t="n">
+      <c r="AT31" t="n">
         <v>53.974125</v>
       </c>
-      <c r="AT31" t="n">
+      <c r="AU31" t="n">
         <v>-0.074613</v>
       </c>
-      <c r="AU31" t="n">
+      <c r="AV31" t="n">
         <v>0.11938</v>
       </c>
-      <c r="AV31" t="n">
+      <c r="AW31" t="n">
+        <v>-0.72538577</v>
+      </c>
+      <c r="AX31" t="n">
         <v>0.171675</v>
       </c>
-      <c r="AW31" t="n">
+      <c r="AY31" t="n">
         <v>1900.90273711537</v>
       </c>
-      <c r="AX31" t="n">
+      <c r="AZ31" t="n">
         <v>314.484004260083</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -5405,32 +5597,32 @@
         <v>0</v>
       </c>
       <c r="AG32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH32" t="n">
         <v>2174.81221062854</v>
       </c>
-      <c r="AH32" t="n">
+      <c r="AI32" t="n">
         <v>353.307686692788</v>
       </c>
-      <c r="AI32" t="n">
+      <c r="AJ32" t="n">
         <v>-3137.15544595861</v>
       </c>
-      <c r="AJ32" t="n">
+      <c r="AK32" t="n">
         <v>-1613.56043146059</v>
       </c>
-      <c r="AK32" t="n">
+      <c r="AL32" t="n">
         <v>-155.593128607218</v>
       </c>
-      <c r="AL32" t="n">
+      <c r="AM32" t="n">
         <v>-74.6998181248039</v>
       </c>
-      <c r="AM32" t="n">
+      <c r="AN32" t="n">
         <v>2252.82029811835</v>
       </c>
-      <c r="AN32" t="n">
+      <c r="AO32" t="n">
         <v>185.110971669093</v>
       </c>
-      <c r="AO32" t="n">
-        <v>0</v>
-      </c>
       <c r="AP32" t="n">
         <v>0</v>
       </c>
@@ -5438,33 +5630,39 @@
         <v>0</v>
       </c>
       <c r="AR32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS32" t="n">
         <v>33.726</v>
       </c>
-      <c r="AS32" t="n">
+      <c r="AT32" t="n">
         <v>55.071</v>
       </c>
-      <c r="AT32" t="n">
+      <c r="AU32" t="n">
         <v>-0.097818</v>
       </c>
-      <c r="AU32" t="n">
+      <c r="AV32" t="n">
         <v>0.0196</v>
       </c>
-      <c r="AV32" t="n">
+      <c r="AW32" t="n">
+        <v>-0.3218514</v>
+      </c>
+      <c r="AX32" t="n">
         <v>0.14805</v>
       </c>
-      <c r="AW32" t="n">
+      <c r="AY32" t="n">
         <v>1922.44609840271</v>
       </c>
-      <c r="AX32" t="n">
+      <c r="AZ32" t="n">
         <v>315.92218268164</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C33" t="n">
         <v>0</v>
@@ -5557,32 +5755,32 @@
         <v>0</v>
       </c>
       <c r="AG33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH33" t="n">
         <v>2209.86888434798</v>
       </c>
-      <c r="AH33" t="n">
+      <c r="AI33" t="n">
         <v>360.094011207122</v>
       </c>
-      <c r="AI33" t="n">
+      <c r="AJ33" t="n">
         <v>-3159.62983931872</v>
       </c>
-      <c r="AJ33" t="n">
+      <c r="AK33" t="n">
         <v>-1630.44318757033</v>
       </c>
-      <c r="AK33" t="n">
+      <c r="AL33" t="n">
         <v>-154.39609561683</v>
       </c>
-      <c r="AL33" t="n">
+      <c r="AM33" t="n">
         <v>-75.3445521061983</v>
       </c>
-      <c r="AM33" t="n">
+      <c r="AN33" t="n">
         <v>2275.41350405558</v>
       </c>
-      <c r="AN33" t="n">
+      <c r="AO33" t="n">
         <v>185.573749098265</v>
       </c>
-      <c r="AO33" t="n">
-        <v>0</v>
-      </c>
       <c r="AP33" t="n">
         <v>0</v>
       </c>
@@ -5590,33 +5788,39 @@
         <v>0</v>
       </c>
       <c r="AR33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS33" t="n">
         <v>34.295</v>
       </c>
-      <c r="AS33" t="n">
+      <c r="AT33" t="n">
         <v>56.3688</v>
       </c>
-      <c r="AT33" t="n">
+      <c r="AU33" t="n">
         <v>-0.082501</v>
       </c>
-      <c r="AU33" t="n">
-        <v>0</v>
-      </c>
       <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX33" t="n">
         <v>0.124425</v>
       </c>
-      <c r="AW33" t="n">
+      <c r="AY33" t="n">
         <v>1947.6580287153</v>
       </c>
-      <c r="AX33" t="n">
+      <c r="AZ33" t="n">
         <v>318.390398374467</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C34" t="n">
         <v>0</v>
@@ -5709,32 +5913,32 @@
         <v>0</v>
       </c>
       <c r="AG34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH34" t="n">
         <v>2244.32384906585</v>
       </c>
-      <c r="AH34" t="n">
+      <c r="AI34" t="n">
         <v>368.198902119206</v>
       </c>
-      <c r="AI34" t="n">
+      <c r="AJ34" t="n">
         <v>-3194.33758142116</v>
       </c>
-      <c r="AJ34" t="n">
+      <c r="AK34" t="n">
         <v>-1647.42314255416</v>
       </c>
-      <c r="AK34" t="n">
+      <c r="AL34" t="n">
         <v>-154.659688545149</v>
       </c>
-      <c r="AL34" t="n">
+      <c r="AM34" t="n">
         <v>-75.6395254520747</v>
       </c>
-      <c r="AM34" t="n">
+      <c r="AN34" t="n">
         <v>2290.2192580238</v>
       </c>
-      <c r="AN34" t="n">
+      <c r="AO34" t="n">
         <v>186.037683471011</v>
       </c>
-      <c r="AO34" t="n">
-        <v>0</v>
-      </c>
       <c r="AP34" t="n">
         <v>0</v>
       </c>
@@ -5742,24 +5946,30 @@
         <v>0</v>
       </c>
       <c r="AR34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS34" t="n">
         <v>34.837</v>
       </c>
-      <c r="AS34" t="n">
+      <c r="AT34" t="n">
         <v>57.2526</v>
       </c>
-      <c r="AT34" t="n">
+      <c r="AU34" t="n">
         <v>-0.067184</v>
       </c>
-      <c r="AU34" t="n">
-        <v>0</v>
-      </c>
       <c r="AV34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX34" t="n">
         <v>0.1008</v>
       </c>
-      <c r="AW34" t="n">
+      <c r="AY34" t="n">
         <v>1974.82326081265</v>
       </c>
-      <c r="AX34" t="n">
+      <c r="AZ34" t="n">
         <v>322.559389434187</v>
       </c>
     </row>

</xml_diff>